<commit_message>
Auto update excel file
</commit_message>
<xml_diff>
--- a/all_grants.xlsx
+++ b/all_grants.xlsx
@@ -489,676 +489,10 @@
       <c r="B2" s="1" t="inlineStr"/>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>EoI - For Empanelment of agencies for Impact Assessment/ Evaluation Servic...</t>
+          <t>RFP - Onboarding Agency for Revamping Assam LMIS Dashboard</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Small Industries Development Bank of India (SIDBI) | India
-International Development - EoI - For Empanelment of agencies for Impact Assessment/ Evaluation Services under Programmes for Development and Impact, Small Industries Development Bank of India (SIDBI), India - DevNetJobsIndia.org
-Jobseekers ... Read More</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>• Please      note that all the information required as per the documents required for      responding to EOI needs to be provided. Incomplete information in these      areas may lead to non-selection.
-Modification      And/ Or Withdrawal of documents:
-Documents once submitted will      be treated as final and no further correspondence will be entertained. No      document shall be modified after the deadline for submission of documents      in response to the EOI. Also, no Respondent shall be allowed to withdraw      any document, if the Respondent happens to be a successful      Respondent.
-SIDBI      has the right to reject any or all documents received without assigning      any reason whatsoever.
-NOTE:
-SIDBI SHALL NOT BE RESPONSIBLE FOR NON-RECEIPT / NON-DELIVERY OF THE DOCUMENTS DUE TO ANY REASON, WHATSOEVER.
-Critical Information
-Events
-Particular / Date and Time
-Tender No
-SIDBI/REOI/68279
-Tender Issue Date
-13/02/2026
-Last date for seeking Clarification on EOI document
-20/02/2026
-All queries relating to the EoI must be in writing only   and to be sent via
-email on.
-pdi@sidbi.in
-and
-mayankp@sidbi.in
-Pre EOI meeting
-25/02/2026
-The meeting shall be virtual / online over MS Teams Call.   Meeting Link will be shared separately to all the bidder
-Last date for submission of EoI
-06/03/2026
-Bids to submitted through email only at:
-pdi@sidbi.in
-and
-mayankp@sidbi.in
-Independent External Monitor
-Shri Sanjay Kumar Srivastava, IAS (Retd.),
-Apartment T-6 B,
-Windsor Court, DLF Phase-IV
-Gurgaon-122009
-Mobile No-9910059472
-E-mail:
-sksrivastava7854@rediffmail.com
-Dr. Parvez Hayat, IPS (Retd.),
-B-4/69- A, Safdarjung Enclave
-New Delhi-110029
-Mobile-9810134469
-E-Mail:
-phayatips@gmail.com
-• Contact details of SIDBI officials
-Shri Mohammed Adil Ahsan
-Asst. General Manager,
-Programmes for Development &amp; Impact [PDI]
-SIDBI Tower, 15, Ashok Marg, Lucknow – 226001
-Ph: 0522-4261631
-Email:
-mdadil@sidbi.in
-Shri Mayank Prakash
-Theme Leader – Monitoring &amp; Evaluation
-Programmes for Development &amp; Impact [PDI]
-SIDBI Tower, 15, Ashok Marg, Lucknow – 226001
-Ph: 0522 - 4259 626
-Email
-mayankp@sidbi.in
-For detailed information, please check the complete version of the EoI attached below.
-Download Attachment:
-EOI for empanelment of Imapact assesment agencies_1202026.pdf
-View Similar Jobs:
-Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
-Subscribe
-Apply by:
-06 Mar 2026
-Access all the jobs and get ahead!
-Subscribe to Value Membership Now!
-Subscribe
-Premium Jobs
-Post your premium jobs here
-Associate – Finance and Operations
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-05 Apr 2026
-Lead-Finance &amp; Compliance
-Marathwada Navnirman Lokayat (Manavlok)
-Location:
-Maharashtra
-Apply by:
-03 Apr 2026
-Sector Experts
-Academy of Management Studies (AMS)
-Location:
-India
-Apply by:
-31 Mar 2026
-Junior Research Technicians / Senior Project Asso...
-Starshield Security Solution Pvt.Ltd
-Location:
-Uttar Pradesh
-Apply by:
-30 Mar 2026
-Agriculture Research Development Officer / Projec...
-Starshield Security Solution Pvt.Ltd
-Location:
-Uttar Pradesh
-Apply by:
-30 Mar 2026
-Specialist - Grants
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-21 Mar 2026
-Specialist – Communication
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-19 Mar 2026
-Specialist – Financial Management and Compliance
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-13 Mar 2026
-Associate (Programme Management)
-Indian Institute For Human Settlements (Iihs)
-Location:
-Karnataka
-Apply by:
-07 Mar 2026
-Chief Programs Officer for Project Potential
-Project Potential
-Location:
-Bihar
-Apply by:
-11 Mar 2026
-Latest Jobs
-Post your highlighted jobs here
-Design and Readiness Lead
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Program Manager – AI Skilling Initiative
-SwaTaleem Foundation
-Location:
-Haryana
-Apply by:
-05 Apr 2026
-Communications Lead
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
-Jobseekers
-Register
-Login
-Subscribe to Value Membership
-Broadcast Resume
-Contact Us
-Recruiters
-Recruiters Zone
-Post a Free Job
-Post a Highlighted Job (With Logo)
-Post a Highlighted Job (Without Logo)
-Post a Premium Job
-More Job Posting Options
-Rates
-Contact Us
-Advertisers
-Networks
-Advertise Your Banner
-Submit Events &amp; Notices
-© 2025 M-Power Jobs. All rights reserved.
-Disclaimer
-Privacy Policy
-Terms &amp; Conditions
-Powered by
-Recruitment Exchange</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>Governance, Learning</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t>06-03-2026</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287084</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>DevNetJobsIndia</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr"/>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>RFP- #2026-IN-01- Agency for economic Impact Analysis</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>PATH | Delhi
-International Development - RFP- #2026-IN-01- Agency for economic Impact Analysis, PATH, Delhi - DevNetJobsIndia.org
-Jobseekers:
-Login
-|
-Register
-Home
-Value Membership
-Broadcast Resume
-RFPs/Tenders
-Search Jobs
-Events
-Jobseekers:
-Login
-|
-Register
-Jobseekers Login
-Jobseekers Register
-Job ... Read More</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>• Job Email ID:
-rfpindia(at)path.org
-Download Attachment:
-Request for Proposal - RFP#2026-IN-01- Agency for economic Impact Analysis.doc
-View Similar Jobs:
-Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
-Subscribe
-Apply by:
-07 Mar 2026
-Access all the jobs and get ahead!
-Subscribe to Value Membership Now!
-Subscribe
-Premium Jobs
-Post your premium jobs here
-Associate – Finance and Operations
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-05 Apr 2026
-Lead-Finance &amp; Compliance
-Marathwada Navnirman Lokayat (Manavlok)
-Location:
-Maharashtra
-Apply by:
-03 Apr 2026
-Sector Experts
-Academy of Management Studies (AMS)
-Location:
-India
-Apply by:
-31 Mar 2026
-Junior Research Technicians / Senior Project Asso...
-Starshield Security Solution Pvt.Ltd
-Location:
-Uttar Pradesh
-Apply by:
-30 Mar 2026
-Agriculture Research Development Officer / Projec...
-Starshield Security Solution Pvt.Ltd
-Location:
-Uttar Pradesh
-Apply by:
-30 Mar 2026
-Specialist - Grants
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-21 Mar 2026
-Specialist – Communication
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-19 Mar 2026
-Specialist – Financial Management and Compliance
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-13 Mar 2026
-Associate (Programme Management)
-Indian Institute For Human Settlements (Iihs)
-Location:
-Karnataka
-Apply by:
-07 Mar 2026
-Chief Programs Officer for Project Potential
-Project Potential
-Location:
-Bihar
-Apply by:
-11 Mar 2026
-Latest Jobs
-Post your highlighted jobs here
-Design and Readiness Lead
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Program Manager – AI Skilling Initiative
-SwaTaleem Foundation
-Location:
-Haryana
-Apply by:
-05 Apr 2026
-Communications Lead
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
-Jobseekers
-Register
-Login
-Subscribe to Value Membership
-Broadcast Resume
-Contact Us
-Recruiters
-Recruiters Zone
-Post a Free Job
-Post a Highlighted Job (With Logo)
-Post a Highlighted Job (Without Logo)
-Post a Premium Job
-More Job Posting Options
-Rates
-Contact Us
-Advertisers
-Networks
-Advertise Your Banner
-Submit Events &amp; Notices
-© 2025 M-Power Jobs. All rights reserved.
-Disclaimer
-Privacy Policy
-Terms &amp; Conditions
-Powered by
-Recruitment Exchange</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="G3" s="1" t="inlineStr">
-        <is>
-          <t>07-03-2026</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287460</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>DevNetJobsIndia</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr"/>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Associate (Programme Management)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Indian Institute For Human Settlements (Iihs) | Karnataka
-International Development - Associate (Programme Management), Indian Institute For Human Settlements (Iihs), Karnataka - DevNetJobsIndia.org
-Jobseekers:
-Login
-|
-Register
-Home
-Value Membership
-Broadcast Resume
-RFPs/Tenders
-Search Jobs
-Events ... Read More</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>• IIHS is an equal opportunity employer that encourages women, people with disabilities and those from economically and socially excluded communities with the requisite skills and qualifications to apply for positions.
-• To apply
-If you are interested in exploring this opportunity with us, please fill the online
-application form
-by clicking here. (You can also click on the “
-Apply Now
-” button at the end of the Job Description displayed on the website).
-Contact
-Please write to us at
-hr@iihs.co.in
-if you need any clarifications while filling the online application form.
-• Job Email ID:
-hr(at)iihs.co.in
-Download Attachment:
-Associate-Programme-Management-–-ASSURE-Lighthouse-Projects.pdf
-View Similar Jobs:
-Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
-Subscribe
-Apply by:
-07 Mar 2026
-Access all the jobs and get ahead!
-Subscribe to Value Membership Now!
-Subscribe
-Premium Jobs
-Post your premium jobs here
-Associate – Finance and Operations
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-05 Apr 2026
-Lead-Finance &amp; Compliance
-Marathwada Navnirman Lokayat (Manavlok)
-Location:
-Maharashtra
-Apply by:
-03 Apr 2026
-Sector Experts
-Academy of Management Studies (AMS)
-Location:
-India
-Apply by:
-31 Mar 2026
-Junior Research Technicians / Senior Project Asso...
-Starshield Security Solution Pvt.Ltd
-Location:
-Uttar Pradesh
-Apply by:
-30 Mar 2026
-Agriculture Research Development Officer / Projec...
-Starshield Security Solution Pvt.Ltd
-Location:
-Uttar Pradesh
-Apply by:
-30 Mar 2026
-Specialist - Grants
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-21 Mar 2026
-Specialist – Communication
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-19 Mar 2026
-Specialist – Financial Management and Compliance
-Financial Management Service Foundation (FMSF)
-Location:
-Uttar Pradesh
-Apply by:
-13 Mar 2026
-Associate (Programme Management)
-Indian Institute For Human Settlements (Iihs)
-Location:
-Karnataka
-Apply by:
-07 Mar 2026
-Chief Programs Officer for Project Potential
-Project Potential
-Location:
-Bihar
-Apply by:
-11 Mar 2026
-Latest Jobs
-Post your highlighted jobs here
-Design and Readiness Lead
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Program Manager – AI Skilling Initiative
-SwaTaleem Foundation
-Location:
-Haryana
-Apply by:
-05 Apr 2026
-Communications Lead
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
-Jobseekers
-Register
-Login
-Subscribe to Value Membership
-Broadcast Resume
-Contact Us
-Recruiters
-Recruiters Zone
-Post a Free Job
-Post a Highlighted Job (With Logo)
-Post a Highlighted Job (Without Logo)
-Post a Premium Job
-More Job Posting Options
-Rates
-Contact Us
-Advertisers
-Networks
-Advertise Your Banner
-Submit Events &amp; Notices
-© 2025 M-Power Jobs. All rights reserved.
-Disclaimer
-Privacy Policy
-Terms &amp; Conditions
-Powered by
-Recruitment Exchange</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>07-03-2026</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=285747</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>DevNetJobsIndia</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr"/>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>RFP - Onboarding Agency for Revamping Assam LMIS Dashboard</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>PATH | Assam
 International Development - RFP - Onboarding Agency for Revamping Assam LMIS Dashboard, PATH, Assam - DevNetJobsIndia.org
@@ -1180,7 +514,7 @@
 Jobseekers Registe ... Read More</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>• 3.2. Commercial contracting terms and conditions will be negotiated with the successful supplier at the end of the selection process.
 3.3. By submitting a proposal, the supplier confirms their agreement to abide by the RFP terms and PATH policies, including the
@@ -1335,6 +669,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -1353,36 +717,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -1410,41 +744,41 @@
 Recruitment Exchange</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>07-03-2026</t>
         </is>
       </c>
-      <c r="H5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" s="1" t="inlineStr">
+      <c r="H2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287335</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>DevNetJobsIndia</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr"/>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>RFQ: Construction of New gated check dams, De-siltation, and retrofitting ...</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>WaterAid India | Telangana
-International Development - RFQ: Construction of New gated check dams, De-siltation, and retrofitting of check dam in 6 villages, WaterAid India, Telangana - DevNetJobsIndia.org
+      <c r="B3" s="1" t="inlineStr"/>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>RFP- #2026-IN-01- Agency for economic Impact Analysis</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>PATH | Delhi
+International Development - RFP- #2026-IN-01- Agency for economic Impact Analysis, PATH, Delhi - DevNetJobsIndia.org
 Jobseekers:
 Login
 |
@@ -1454,20 +788,27 @@
 Broadcast Resume
 RFPs/Tenders
 Search Jobs
-E ... Read More</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+Events
+Jobseekers:
+Login
+|
+Register
+Jobseekers Login
+Jobseekers Register
+Job ... Read More</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>• Job Email ID:
-WAIProcurementAP(at)wateraid.org
+rfpindia(at)path.org
 Download Attachment:
-Tender Notice-15 check dams-Jalsankalp-19.02.26_compressed.pdf
+Request for Proposal - RFP#2026-IN-01- Agency for economic Impact Analysis.doc
 View Similar Jobs:
 Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
 Subscribe
 Apply by:
-08 Mar 2026
+07 Mar 2026
 Access all the jobs and get ahead!
 Subscribe to Value Membership Now!
 Subscribe
@@ -1535,6 +876,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -1553,36 +924,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -1610,38 +951,449 @@
 Recruitment Exchange</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>07-03-2026</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287460</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>DevNetJobsIndia</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr"/>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Associate (Programme Management)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Indian Institute For Human Settlements (Iihs) | Karnataka
+International Development - Associate (Programme Management), Indian Institute For Human Settlements (Iihs), Karnataka - DevNetJobsIndia.org
+Jobseekers:
+Login
+|
+Register
+Home
+Value Membership
+Broadcast Resume
+RFPs/Tenders
+Search Jobs
+Events ... Read More</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>• IIHS is an equal opportunity employer that encourages women, people with disabilities and those from economically and socially excluded communities with the requisite skills and qualifications to apply for positions.
+• To apply
+If you are interested in exploring this opportunity with us, please fill the online
+application form
+by clicking here. (You can also click on the “
+Apply Now
+” button at the end of the Job Description displayed on the website).
+Contact
+Please write to us at
+hr@iihs.co.in
+if you need any clarifications while filling the online application form.
+• Job Email ID:
+hr(at)iihs.co.in
+Download Attachment:
+Associate-Programme-Management-–-ASSURE-Lighthouse-Projects.pdf
+View Similar Jobs:
+Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
+Subscribe
+Apply by:
+07 Mar 2026
+Access all the jobs and get ahead!
+Subscribe to Value Membership Now!
+Subscribe
+Premium Jobs
+Post your premium jobs here
+Associate – Finance and Operations
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+05 Apr 2026
+Lead-Finance &amp; Compliance
+Marathwada Navnirman Lokayat (Manavlok)
+Location:
+Maharashtra
+Apply by:
+03 Apr 2026
+Sector Experts
+Academy of Management Studies (AMS)
+Location:
+India
+Apply by:
+31 Mar 2026
+Junior Research Technicians / Senior Project Asso...
+Starshield Security Solution Pvt.Ltd
+Location:
+Uttar Pradesh
+Apply by:
+30 Mar 2026
+Agriculture Research Development Officer / Projec...
+Starshield Security Solution Pvt.Ltd
+Location:
+Uttar Pradesh
+Apply by:
+30 Mar 2026
+Specialist - Grants
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+21 Mar 2026
+Specialist – Communication
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+19 Mar 2026
+Specialist – Financial Management and Compliance
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+13 Mar 2026
+Associate (Programme Management)
+Indian Institute For Human Settlements (Iihs)
+Location:
+Karnataka
+Apply by:
+07 Mar 2026
+Chief Programs Officer for Project Potential
+Project Potential
+Location:
+Bihar
+Apply by:
+11 Mar 2026
+Latest Jobs
+Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
+Design and Readiness Lead
+SwaTaleem Foundation
+Location:
+Delhi
+Apply by:
+05 Apr 2026
+Program Manager – AI Skilling Initiative
+SwaTaleem Foundation
+Location:
+Haryana
+Apply by:
+05 Apr 2026
+Communications Lead
+SwaTaleem Foundation
+Location:
+Delhi
+Apply by:
+05 Apr 2026
+Jobseekers
+Register
+Login
+Subscribe to Value Membership
+Broadcast Resume
+Contact Us
+Recruiters
+Recruiters Zone
+Post a Free Job
+Post a Highlighted Job (With Logo)
+Post a Highlighted Job (Without Logo)
+Post a Premium Job
+More Job Posting Options
+Rates
+Contact Us
+Advertisers
+Networks
+Advertise Your Banner
+Submit Events &amp; Notices
+© 2025 M-Power Jobs. All rights reserved.
+Disclaimer
+Privacy Policy
+Terms &amp; Conditions
+Powered by
+Recruitment Exchange</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>07-03-2026</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=285747</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>DevNetJobsIndia</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr"/>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>RFQ: Construction of New gated check dams, De-siltation, and retrofitting ...</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>WaterAid India | Telangana
+International Development - RFQ: Construction of New gated check dams, De-siltation, and retrofitting of check dam in 6 villages, WaterAid India, Telangana - DevNetJobsIndia.org
+Jobseekers:
+Login
+|
+Register
+Home
+Value Membership
+Broadcast Resume
+RFPs/Tenders
+Search Jobs
+E ... Read More</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>• Job Email ID:
+WAIProcurementAP(at)wateraid.org
+Download Attachment:
+Tender Notice-15 check dams-Jalsankalp-19.02.26_compressed.pdf
+View Similar Jobs:
+Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
+Subscribe
+Apply by:
+08 Mar 2026
+Access all the jobs and get ahead!
+Subscribe to Value Membership Now!
+Subscribe
+Premium Jobs
+Post your premium jobs here
+Associate – Finance and Operations
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+05 Apr 2026
+Lead-Finance &amp; Compliance
+Marathwada Navnirman Lokayat (Manavlok)
+Location:
+Maharashtra
+Apply by:
+03 Apr 2026
+Sector Experts
+Academy of Management Studies (AMS)
+Location:
+India
+Apply by:
+31 Mar 2026
+Junior Research Technicians / Senior Project Asso...
+Starshield Security Solution Pvt.Ltd
+Location:
+Uttar Pradesh
+Apply by:
+30 Mar 2026
+Agriculture Research Development Officer / Projec...
+Starshield Security Solution Pvt.Ltd
+Location:
+Uttar Pradesh
+Apply by:
+30 Mar 2026
+Specialist - Grants
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+21 Mar 2026
+Specialist – Communication
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+19 Mar 2026
+Specialist – Financial Management and Compliance
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+13 Mar 2026
+Associate (Programme Management)
+Indian Institute For Human Settlements (Iihs)
+Location:
+Karnataka
+Apply by:
+07 Mar 2026
+Chief Programs Officer for Project Potential
+Project Potential
+Location:
+Bihar
+Apply by:
+11 Mar 2026
+Latest Jobs
+Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
+Design and Readiness Lead
+SwaTaleem Foundation
+Location:
+Delhi
+Apply by:
+05 Apr 2026
+Program Manager – AI Skilling Initiative
+SwaTaleem Foundation
+Location:
+Haryana
+Apply by:
+05 Apr 2026
+Communications Lead
+SwaTaleem Foundation
+Location:
+Delhi
+Apply by:
+05 Apr 2026
+Jobseekers
+Register
+Login
+Subscribe to Value Membership
+Broadcast Resume
+Contact Us
+Recruiters
+Recruiters Zone
+Post a Free Job
+Post a Highlighted Job (With Logo)
+Post a Highlighted Job (Without Logo)
+Post a Premium Job
+More Job Posting Options
+Rates
+Contact Us
+Advertisers
+Networks
+Advertise Your Banner
+Submit Events &amp; Notices
+© 2025 M-Power Jobs. All rights reserved.
+Disclaimer
+Privacy Policy
+Terms &amp; Conditions
+Powered by
+Recruitment Exchange</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>08-03-2026</t>
         </is>
       </c>
-      <c r="H6" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" s="1" t="inlineStr">
+      <c r="H5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287784</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>DevNetJobsIndia</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr"/>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr"/>
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>RFP - Final Evaluation of the Bhoomi Ka Programme</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Deutsche Welthungerhilfe | India
 International Development - RFP - Final Evaluation of the Bhoomi Ka Programme, Deutsche Welthungerhilfe, India - DevNetJobsIndia.org
@@ -1662,7 +1414,7 @@
 Jobs ... Read More</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>• INTRODUCTION AND CONTEXT
 Country:
@@ -1792,6 +1544,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -1810,36 +1592,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -1867,49 +1619,48 @@
 Recruitment Exchange</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="G7" s="1" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>08-03-2026</t>
         </is>
       </c>
-      <c r="H7" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="I7" s="1" t="inlineStr">
+      <c r="H6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
         <is>
           <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287384</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>DevNetJobsIndia</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr"/>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>RFP For The Contractors To Procure, Build, Install, Supply Chlorine Tablet...</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr"/>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>RFP For Selection of an Implementation Support Agency (Isa) For Capacity B...</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>EAII Advisors Pvt Ltd | Andhra Pradesh
-International Development - RFP For The Contractors To Procure, Build, Install, Supply Chlorine Tablets, Operate And Maintain Tablet-Based In Line Chlorination Devices, EAII Advisors Pvt Ltd, Andhra Pradesh - DevNetJobsIndia.org
+International Development - RFP For Selection of an Implementation Support Agency (Isa) For Capacity Building Of Community Leaders To Conduct Community Engagement Activities, EAII Advisors Pvt Ltd, Andhra Pradesh - DevNetJobsIndia.org
 Jobseekers:
 Login
 |
-Register
-Ho ... Read More</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
+Regis ... Read More</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>• Proposal Requirements
 1. Company Background and Details
@@ -1919,9 +1670,9 @@
 Kindly fill in the column “Bidder Response”. The current inputs are guiding inputs or choices for answers. Kindly fill in accordingly.
 For detailed information, please check the complete version of the RFP attached below.
 Download Attachment:
-Standalone IC RFP Technical Evaluation Response Template.docx
+Standalone ISA RFP Technical Evaluation Response Template (1).docx
 Download Attachment:
-Telugu_Standalone IC RFP Technical Evaluation Response Template.docx
+Telugu_Standalone ISA RFP Technical Evaluation Response Template.docx
 View Similar Jobs:
 Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
 Subscribe
@@ -1994,6 +1745,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -2012,36 +1793,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -2069,9 +1820,59 @@
 Recruitment Exchange</t>
         </is>
       </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>Governance, Learning</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>09-03-2026</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=285950</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DevNetJobsIndia</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr"/>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>RFP - Early-Stage Impact Assessment-CDRI SWP 23-26</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Coalition for Disaster Resilient Infrastructure (CDRI) | India
+International Development - RFP - Early-Stage Impact Assessment-CDRI SWP 23-26, Coalition for Disaster Resilient Infrastructure (CDRI), India - DevNetJobsIndia.org
+Jobseekers:
+Login
+|
+Register
+Home
+Value Membership
+Broadcast Resume
+RFPs ... Read More</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Climate, Governance</t>
         </is>
       </c>
       <c r="G8" s="1" t="inlineStr">
@@ -2080,11 +1881,11 @@
         </is>
       </c>
       <c r="H8" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I8" s="1" t="inlineStr">
         <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=285949</t>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287093</t>
         </is>
       </c>
     </row>
@@ -2192,6 +1993,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -2210,36 +2041,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -2278,7 +2079,7 @@
         </is>
       </c>
       <c r="H9" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
@@ -2295,70 +2096,21 @@
       <c r="B10" s="1" t="inlineStr"/>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>RFP - Early-Stage Impact Assessment-CDRI SWP 23-26</t>
+          <t>RFP For The Contractors To Procure, Build, Install, Supply Chlorine Tablet...</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Coalition for Disaster Resilient Infrastructure (CDRI) | India
-International Development - RFP - Early-Stage Impact Assessment-CDRI SWP 23-26, Coalition for Disaster Resilient Infrastructure (CDRI), India - DevNetJobsIndia.org
+          <t>EAII Advisors Pvt Ltd | Andhra Pradesh
+International Development - RFP For The Contractors To Procure, Build, Install, Supply Chlorine Tablets, Operate And Maintain Tablet-Based In Line Chlorination Devices, EAII Advisors Pvt Ltd, Andhra Pradesh - DevNetJobsIndia.org
 Jobseekers:
 Login
 |
 Register
-Home
-Value Membership
-Broadcast Resume
-RFPs ... Read More</t>
+Ho ... Read More</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>Climate, Governance</t>
-        </is>
-      </c>
-      <c r="G10" s="1" t="inlineStr">
-        <is>
-          <t>09-03-2026</t>
-        </is>
-      </c>
-      <c r="H10" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="I10" s="1" t="inlineStr">
-        <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287093</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>DevNetJobsIndia</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr"/>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>RFP For Selection of an Implementation Support Agency (Isa) For Capacity B...</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>EAII Advisors Pvt Ltd | Andhra Pradesh
-International Development - RFP For Selection of an Implementation Support Agency (Isa) For Capacity Building Of Community Leaders To Conduct Community Engagement Activities, EAII Advisors Pvt Ltd, Andhra Pradesh - DevNetJobsIndia.org
-Jobseekers:
-Login
-|
-Regis ... Read More</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>• Proposal Requirements
 1. Company Background and Details
@@ -2368,9 +2120,9 @@
 Kindly fill in the column “Bidder Response”. The current inputs are guiding inputs or choices for answers. Kindly fill in accordingly.
 For detailed information, please check the complete version of the RFP attached below.
 Download Attachment:
-Standalone ISA RFP Technical Evaluation Response Template (1).docx
+Standalone IC RFP Technical Evaluation Response Template.docx
 Download Attachment:
-Telugu_Standalone ISA RFP Technical Evaluation Response Template.docx
+Telugu_Standalone IC RFP Technical Evaluation Response Template.docx
 View Similar Jobs:
 Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
 Subscribe
@@ -2443,6 +2195,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -2461,36 +2243,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -2518,38 +2270,38 @@
 Recruitment Exchange</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>Governance, Learning</t>
-        </is>
-      </c>
-      <c r="G11" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>09-03-2026</t>
         </is>
       </c>
-      <c r="H11" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="I11" s="1" t="inlineStr">
-        <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=285950</t>
+      <c r="H10" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=285949</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>DevNetJobsIndia</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr"/>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr"/>
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>RFP - for Supply of Skill Lab Items</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>TeamLease Foundation | India
 International Development - RFP - for Supply of Skill Lab Items, TeamLease Foundation, India - DevNetJobsIndia.org
@@ -2571,7 +2323,7 @@
 Jobseeker ... Read More</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>• Technical Bid Submission Link-
 https://forms.gle/V9iy35ddb4kWEb468
@@ -2678,6 +2430,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -2696,36 +2478,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -2753,44 +2505,44 @@
 Recruitment Exchange</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="G12" s="1" t="inlineStr">
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>11-03-2026</t>
         </is>
       </c>
-      <c r="H12" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="I12" s="1" t="inlineStr">
+      <c r="H11" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
         <is>
           <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287613</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>DevNetJobsIndia</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr"/>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr"/>
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>RFP - Study On SC-DMPA In Rajasthan- Clients And Providers Perspectives On...</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Centre For Community Economics And Development Consultants Society- CECOEDECON | Jaipur, Rajasthan
 International Development - RFP - Study On SC-DMPA In Rajasthan- Clients And Providers Perspectives On SC-DMPA In Rajasthan, Centre For Community Economics And Development Consultants Society- CECOEDE ... Read More</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>• Despite India’s achievement of replacement-level fertility, unmet need for contraception—particularly for spacing methods—remains substantial, with modern contraceptive use at 56.4% (2019–21), highlighting persistent gaps in access and choice, especially among vulnerable populations. Expanding the contraceptive method mix through innovative, user-centred approaches is therefore essential to meeting national commitments under FP2030 and the Sustainable Development Goals. In this context, the Government of India’s introduction of subcutaneous DMPA (DMPA-SC) as a self-care option under the National Family Planning Programme in 2023 represents a strategic step toward enhancing women’s autonomy, privacy, and convenience in contraceptive use. Global and national evidence indicates strong feasibility and acceptability of self-administered DMPA-SC among both users and providers; however, successful implementation requires an in-depth understanding of user experiences and health system readiness. This study, to be conducted in Jaipur-1, Jaisalmer and Sawai Madhopur districts of Rajasthan, aims to examine the perspectives &amp; experience of current SC-DMPA users and explore healthcare providers’ views on enabling and generating actionable evidence to inform effective scale-up of SC-DMPA within India’s public health system.
 CECOEDECON, with support from UNFPA, is implementing the roll-out of subcutaneous DMPA (SC-DMPA) in selected pilot districts of Rajasthan in the public health facilities, in collaboration with the Department of Health &amp; Family Welfare, Government of Rajasthan.
@@ -2925,6 +2677,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -2943,36 +2725,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -3000,38 +2752,38 @@
 Recruitment Exchange</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>Learning</t>
         </is>
       </c>
-      <c r="G13" s="1" t="inlineStr">
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>11-03-2026</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="I13" s="1" t="inlineStr">
+      <c r="H12" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
         <is>
           <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287322</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>DevNetJobsIndia</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr"/>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr"/>
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>SOW - Engagement of a Public Relations (PR) Agency on Retainer</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Room to Read India | India
 International Development - SOW - Engagement of a Public Relations (PR) Agency on Retainer, Room to Read India, India - DevNetJobsIndia.org
@@ -3052,7 +2804,7 @@
 Job ... Read More</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>• Scope of Work (SOW)
 Engagement of a Public Relations (PR) Agency on Retainer
@@ -3182,6 +2934,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -3200,36 +2982,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -3257,14 +3009,227 @@
 Recruitment Exchange</t>
         </is>
       </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>Governance, Learning</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>12-03-2026</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287648</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>DevNetJobsIndia</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr"/>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>RFP - for Internal Audit</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>India HIV/AIDS Alliance (Alliance India) | Delhi
+International Development - RFP - for Internal Audit, India HIV/AIDS Alliance (Alliance India), Delhi - DevNetJobsIndia.org
+Jobseekers:
+Login
+|
+Register
+Home
+Value Membership
+Broadcast Resume
+RFPs/Tenders
+Search Jobs
+Events
+Jobseekers:
+Login
+|
+Regist ... Read More</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>• Alliance India reserves the right to reject applications that do not meet eligibility or application submission requirements (as detailed above) without further notice to the applicant. Issuance of this RFP does not constitute an award commitment or a guarantee of business on the part of Alliance India, nor does it commit Alliance India to pay for the costs incurred in submitting the application. Further, Alliance India reserves the right to reject any or all applications received and negotiate separately with an applicant if such action is considered in the best interest of Alliance India/ project.
+iii.
+Queries, Response and Submission
+Queries regarding this RFP will be sent only to procurement@allianceindia.org by March 07, 2026. Alliance India shall collaborate and respond to all meaningful queries from prospective applicants by March 10, 2026. Responses to questions shall be compiled and sent to all the applicants who raised the queries through email only. ALLIANCE INDIA is under no obligation to consider or respond to questions that are not received on time.
+iv.
+• Submission of bids
+The bid has to be submitted in the prescribed format on or before March 13, 2026 by 5 p.m. Indian Standard Time to
+procurement@allianceindia.org
+For the detailed version of the Request for Proposal, please refer to the RFP attached.
+• Job Email ID:
+procurement(at)allianceindia.org
+Download Attachment:
+RFP for Internal Audit - FY 2025-26.doc
+View Similar Jobs:
+Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
+Subscribe
+Apply by:
+13 Mar 2026
+Access all the jobs and get ahead!
+Subscribe to Value Membership Now!
+Subscribe
+Premium Jobs
+Post your premium jobs here
+Associate – Finance and Operations
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+05 Apr 2026
+Lead-Finance &amp; Compliance
+Marathwada Navnirman Lokayat (Manavlok)
+Location:
+Maharashtra
+Apply by:
+03 Apr 2026
+Sector Experts
+Academy of Management Studies (AMS)
+Location:
+India
+Apply by:
+31 Mar 2026
+Junior Research Technicians / Senior Project Asso...
+Starshield Security Solution Pvt.Ltd
+Location:
+Uttar Pradesh
+Apply by:
+30 Mar 2026
+Agriculture Research Development Officer / Projec...
+Starshield Security Solution Pvt.Ltd
+Location:
+Uttar Pradesh
+Apply by:
+30 Mar 2026
+Specialist - Grants
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+21 Mar 2026
+Specialist – Communication
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+19 Mar 2026
+Specialist – Financial Management and Compliance
+Financial Management Service Foundation (FMSF)
+Location:
+Uttar Pradesh
+Apply by:
+13 Mar 2026
+Associate (Programme Management)
+Indian Institute For Human Settlements (Iihs)
+Location:
+Karnataka
+Apply by:
+07 Mar 2026
+Chief Programs Officer for Project Potential
+Project Potential
+Location:
+Bihar
+Apply by:
+11 Mar 2026
+Latest Jobs
+Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
+Design and Readiness Lead
+SwaTaleem Foundation
+Location:
+Delhi
+Apply by:
+05 Apr 2026
+Program Manager – AI Skilling Initiative
+SwaTaleem Foundation
+Location:
+Haryana
+Apply by:
+05 Apr 2026
+Communications Lead
+SwaTaleem Foundation
+Location:
+Delhi
+Apply by:
+05 Apr 2026
+Jobseekers
+Register
+Login
+Subscribe to Value Membership
+Broadcast Resume
+Contact Us
+Recruiters
+Recruiters Zone
+Post a Free Job
+Post a Highlighted Job (With Logo)
+Post a Highlighted Job (Without Logo)
+Post a Premium Job
+More Job Posting Options
+Rates
+Contact Us
+Advertisers
+Networks
+Advertise Your Banner
+Submit Events &amp; Notices
+© 2025 M-Power Jobs. All rights reserved.
+Disclaimer
+Privacy Policy
+Terms &amp; Conditions
+Powered by
+Recruitment Exchange</t>
+        </is>
+      </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>Governance, Learning</t>
+          <t>Learning</t>
         </is>
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>12-03-2026</t>
+          <t>13-03-2026</t>
         </is>
       </c>
       <c r="H14" s="1" t="n">
@@ -3272,7 +3237,7 @@
       </c>
       <c r="I14" s="1" t="inlineStr">
         <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287648</t>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287765</t>
         </is>
       </c>
     </row>
@@ -3415,6 +3380,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -3433,36 +3428,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -3501,7 +3466,7 @@
         </is>
       </c>
       <c r="H15" s="1" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I15" s="1" t="inlineStr">
         <is>
@@ -3518,13 +3483,13 @@
       <c r="B16" s="1" t="inlineStr"/>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>RFP - for Internal Audit</t>
+          <t>ToR - Portfolio-Wide Learning Exercise cum review for the Health Domain</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>India HIV/AIDS Alliance (Alliance India) | Delhi
-International Development - RFP - for Internal Audit, India HIV/AIDS Alliance (Alliance India), Delhi - DevNetJobsIndia.org
+          <t>ChildFund India | India
+International Development - ToR - Portfolio-Wide Learning Exercise cum review for the Health Domain, ChildFund India, India - DevNetJobsIndia.org
 Jobseekers:
 Login
 |
@@ -3538,29 +3503,20 @@
 Jobseekers:
 Login
 |
-Regist ... Read More</t>
+Register ... Read More</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>• Alliance India reserves the right to reject applications that do not meet eligibility or application submission requirements (as detailed above) without further notice to the applicant. Issuance of this RFP does not constitute an award commitment or a guarantee of business on the part of Alliance India, nor does it commit Alliance India to pay for the costs incurred in submitting the application. Further, Alliance India reserves the right to reject any or all applications received and negotiate separately with an applicant if such action is considered in the best interest of Alliance India/ project.
-iii.
-Queries, Response and Submission
-Queries regarding this RFP will be sent only to procurement@allianceindia.org by March 07, 2026. Alliance India shall collaborate and respond to all meaningful queries from prospective applicants by March 10, 2026. Responses to questions shall be compiled and sent to all the applicants who raised the queries through email only. ALLIANCE INDIA is under no obligation to consider or respond to questions that are not received on time.
-iv.
-• Submission of bids
-The bid has to be submitted in the prescribed format on or before March 13, 2026 by 5 p.m. Indian Standard Time to
-procurement@allianceindia.org
-For the detailed version of the Request for Proposal, please refer to the RFP attached.
-• Job Email ID:
-procurement(at)allianceindia.org
+          <t>• Job Email ID:
+centralpurchase2(at)childfundindia.org
 Download Attachment:
-RFP for Internal Audit - FY 2025-26.doc
+TOR  Health Portfolio_23.2.2026.doc
 View Similar Jobs:
 Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
 Subscribe
 Apply by:
-13 Mar 2026
+15 Mar 2026
 Access all the jobs and get ahead!
 Subscribe to Value Membership Now!
 Subscribe
@@ -3628,6 +3584,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -3646,36 +3632,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -3705,20 +3661,20 @@
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>Learning</t>
+          <t>Learning, Safety</t>
         </is>
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>13-03-2026</t>
+          <t>15-03-2026</t>
         </is>
       </c>
       <c r="H16" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287765</t>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287901</t>
         </is>
       </c>
     </row>
@@ -3731,13 +3687,13 @@
       <c r="B17" s="1" t="inlineStr"/>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>ToR - Strategic Review and Forward-Looking Education Strategy Development</t>
+          <t>RFP for Data Collection for Foundational Reading Tool in Odisha</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ChildFund India | India
-International Development - ToR - Strategic Review and Forward-Looking Education Strategy Development, ChildFund India, India - DevNetJobsIndia.org
+          <t>Lords Education and Health Society (LEHS) | Odisha
+International Development - RFP for Data Collection for Foundational Reading Tool in Odisha, Lords Education and Health Society (LEHS), Odisha - DevNetJobsIndia.org
 Jobseekers:
 Login
 |
@@ -3746,20 +3702,36 @@
 Value Membership
 Broadcast Resume
 RFPs/Tenders
-Search Jobs
-Events
-Jobseekers:
-Login
-|
-Registe ... Read More</t>
+Se ... Read More</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>• Job Email ID:
-centralpurchase2(at)childfundindia.org
+          <t>• 4. SCOPE OF WORK
+Summary of Activities
+S.No
+Activity   Description
+Timelines
+1
+Data   Collection: students' reading of textual items   (letters/words/non-words/paragraphs) in Odia &amp; English languages for   Grades 1-8.
+Data       Collection should be completed in   April 2026
+Details of the Activity Below:
+Data Collection: Collect audio data of students reading texts in Odia &amp; English from Grade 1-8
+Total Number of Hours to be collected: ~360 hours for the Odia language
+Total Number of Hours to be collected: ~115 hours for the English language
+• Submission Details
+All proposals to this RFP must be received no later than &lt;15th March 2026&gt;
+.
+The proposal should be submitted only through e-mail in PDF format addressed to the Procurement Team at:
+rfp.lehs@wadhwaniai.org
+. The email's subject line must contain the reference number and title of the RFP: Data Collection for Foundational Reading
+Tool in Odisha  (Name of Partner)
+Any proposals received by Wadhwani-AI after the deadline prescribed in the timeline of this document are liable to be rejected.
+For detailed information, please check the complete version of the RFP attached below
+• Job Email ID:
+rfp.lehs(at)wadhwaniai.org
 Download Attachment:
-ToR for Education.doc
+RFP for Data Collection for Foundational Reading Tool in Odisha.pdf
 View Similar Jobs:
 Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
 Subscribe
@@ -3832,6 +3804,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -3850,36 +3852,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -3909,7 +3881,7 @@
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>Learning, Safety</t>
+          <t>Governance, Learning, Safety</t>
         </is>
       </c>
       <c r="G17" s="1" t="inlineStr">
@@ -3918,11 +3890,11 @@
         </is>
       </c>
       <c r="H17" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I17" s="1" t="inlineStr">
         <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287902</t>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287936</t>
         </is>
       </c>
     </row>
@@ -4095,6 +4067,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -4113,36 +4115,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -4181,7 +4153,7 @@
         </is>
       </c>
       <c r="H18" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I18" s="1" t="inlineStr">
         <is>
@@ -4318,6 +4290,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -4336,36 +4338,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -4404,7 +4376,7 @@
         </is>
       </c>
       <c r="H19" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
@@ -4421,13 +4393,13 @@
       <c r="B20" s="1" t="inlineStr"/>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>ToR - Portfolio-Wide Learning Exercise cum review for the Health Domain</t>
+          <t>ToR - Strategic Review and Forward-Looking Education Strategy Development</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
           <t>ChildFund India | India
-International Development - ToR - Portfolio-Wide Learning Exercise cum review for the Health Domain, ChildFund India, India - DevNetJobsIndia.org
+International Development - ToR - Strategic Review and Forward-Looking Education Strategy Development, ChildFund India, India - DevNetJobsIndia.org
 Jobseekers:
 Login
 |
@@ -4441,7 +4413,7 @@
 Jobseekers:
 Login
 |
-Register ... Read More</t>
+Registe ... Read More</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -4449,7 +4421,7 @@
           <t>• Job Email ID:
 centralpurchase2(at)childfundindia.org
 Download Attachment:
-TOR  Health Portfolio_23.2.2026.doc
+ToR for Education.doc
 View Similar Jobs:
 Was this job of interest to you? Subscribe to Value Membership to get access to similar jobs and hundreds of other member-only jobs.
 Subscribe
@@ -4522,6 +4494,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -4540,36 +4542,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -4608,11 +4580,11 @@
         </is>
       </c>
       <c r="H20" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I20" s="1" t="inlineStr">
         <is>
-          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287901</t>
+          <t>https://www.devnetjobsindia.org/JobDescription.aspx?Job_Id=287902</t>
         </is>
       </c>
     </row>
@@ -4657,7 +4629,7 @@
         </is>
       </c>
       <c r="H21" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I21" s="1" t="inlineStr">
         <is>
@@ -4795,6 +4767,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -4813,36 +4815,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -4881,7 +4853,7 @@
         </is>
       </c>
       <c r="H22" s="1" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I22" s="1" t="inlineStr">
         <is>
@@ -5001,6 +4973,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -5019,36 +5021,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -5087,7 +5059,7 @@
         </is>
       </c>
       <c r="H23" s="1" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I23" s="1" t="inlineStr">
         <is>
@@ -5206,6 +5178,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -5224,36 +5226,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -5292,7 +5264,7 @@
         </is>
       </c>
       <c r="H24" s="1" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I24" s="1" t="inlineStr">
         <is>
@@ -5413,6 +5385,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -5431,36 +5433,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -5499,7 +5471,7 @@
         </is>
       </c>
       <c r="H25" s="1" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I25" s="1" t="inlineStr">
         <is>
@@ -5621,6 +5593,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -5639,36 +5641,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -5707,7 +5679,7 @@
         </is>
       </c>
       <c r="H26" s="1" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I26" s="1" t="inlineStr">
         <is>
@@ -5850,6 +5822,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -5868,36 +5870,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -5936,7 +5908,7 @@
         </is>
       </c>
       <c r="H27" s="1" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I27" s="1" t="inlineStr">
         <is>
@@ -6079,6 +6051,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -6097,36 +6099,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -6165,7 +6137,7 @@
         </is>
       </c>
       <c r="H28" s="1" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I28" s="1" t="inlineStr">
         <is>
@@ -6308,6 +6280,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -6326,36 +6328,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -6394,7 +6366,7 @@
         </is>
       </c>
       <c r="H29" s="1" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I29" s="1" t="inlineStr">
         <is>
@@ -6531,6 +6503,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -6549,36 +6551,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -6617,7 +6589,7 @@
         </is>
       </c>
       <c r="H30" s="1" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I30" s="1" t="inlineStr">
         <is>
@@ -6736,6 +6708,36 @@
 11 Mar 2026
 Latest Jobs
 Post your highlighted jobs here
+RFP for Data Collection for Foundational Reading ...
+Lords Education and Health Society (LEHS)
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Research Scientist – I (Non Medical)
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Project Technical Support - III
+Affordable Quality Health/ACCESS Health Internati...
+Location:
+Odisha
+Apply by:
+15 Mar 2026
+Program Lead- Governance and Gender Justice
+Society for Women's Action and Training Initiativ...
+Location:
+Gujarat
+Apply by:
+25 Mar 2026
+Senior Field Officer Certification Management
+Fairtrade India Project - CSM
+Location:
+Andhra Pradesh
+Apply by:
+15 Mar 2026
 Design and Readiness Lead
 SwaTaleem Foundation
 Location:
@@ -6754,36 +6756,6 @@
 Delhi
 Apply by:
 05 Apr 2026
-Director of International Programmes Impact And P...
-Confidential
-Location:
-Telangana
-Apply by:
-08 Apr 2026
-Organizational Development (OD) Manager
-SwaTaleem Foundation
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-Manager – Monitoring &amp; Evaluation
-Family Planning Association of India (FPA India)
-Location:
-Maharashtra
-Apply by:
-04 Apr 2026
-Officer – Instructional Design and Technical Supp...
-Room to Read India
-Location:
-Delhi
-Apply by:
-05 Apr 2026
-RFP UNW-IND-2026-00002 for Hiring resource agency...
-UN Women
-Location:
-India
-Apply by:
-23 Mar 2026
 Jobseekers
 Register
 Login
@@ -6822,7 +6794,7 @@
         </is>
       </c>
       <c r="H31" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I31" s="1" t="inlineStr">
         <is>

</xml_diff>